<commit_message>
feat: add access plan and fix excel
</commit_message>
<xml_diff>
--- a/public/docs/inscription-equipe.xlsx
+++ b/public/docs/inscription-equipe.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY/MM/DD"/>
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -980,7 +980,7 @@
       <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Date de naissance
-(AAAA/MM/JJ)</t>
+(JJ/MM/AAAA)</t>
         </is>
       </c>
       <c r="E4" s="21" t="inlineStr">

</xml_diff>

<commit_message>
fix: remove prep l2
</commit_message>
<xml_diff>
--- a/public/docs/inscription-equipe.xlsx
+++ b/public/docs/inscription-equipe.xlsx
@@ -881,7 +881,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valeur invalide" error="Choisissez une division dans la liste" type="list">
-      <formula1>Listes!$A$1:$A$49</formula1>
+      <formula1>Listes!$A$1:$A$45</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1598,7 +1598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A49"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1639,306 +1639,278 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>U12 Prep L2</t>
+          <t>U16 Prep L1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>U16 Prep L1</t>
+          <t>U16 Prep L2.1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>U16 Prep L2.1</t>
+          <t>U18 Prep L1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>U16 Prep L2</t>
+          <t>U18 Prep L2.1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>U18 Prep L1</t>
+          <t>Open Prep L1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>U18 Prep L2.1</t>
+          <t>Open Prep L2.1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>U18 Prep L2</t>
+          <t>U12 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Open Prep L1</t>
+          <t>U12 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Open Prep L2.1</t>
+          <t>U16 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Open Prep L2</t>
+          <t>U16 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>U12 Allstar L1</t>
+          <t>U16 Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>U12 Allstar L2</t>
+          <t>U18 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>U16 Allstar L1</t>
+          <t>U18 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>U16 Allstar L2</t>
+          <t>U18 Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>U16 Allstar L3</t>
+          <t>U18 Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>U18 Allstar L1</t>
+          <t>Open Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>U18 Allstar L2</t>
+          <t>Open Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>U18 Allstar L3</t>
+          <t>Open AG Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>U18 Allstar L4</t>
+          <t>Open AG Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Open Allstar L1</t>
+          <t>Open AG Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Open Allstar L2</t>
+          <t>Open AG Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Open AG Allstar L3</t>
+          <t>Open AG Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Open AG Allstar L4</t>
+          <t>Open Coed Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Open AG Allstar L5</t>
+          <t>Open Coed Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Open AG Allstar L6</t>
+          <t>Open Coed Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Open AG Allstar L7</t>
+          <t>Open Coed Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L3</t>
+          <t>Open Coed Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L4</t>
+          <t>Open NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L5</t>
+          <t>Open AG NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L6</t>
+          <t>Open AG NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L7</t>
+          <t>Open AG NT Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Open NT Allstar L2</t>
+          <t>Open AG NT Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L3</t>
+          <t>Open AG NT Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L4</t>
+          <t>Open Coed NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L5</t>
+          <t>Open Coed NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L6</t>
+          <t>Open Coed NT Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L7</t>
+          <t>Open Coed NT Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L3</t>
+          <t>Open Coed NT Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L4</t>
+          <t>Universitaire L2</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
-        <is>
-          <t>Open Coed NT Allstar L5</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Open Coed NT Allstar L6</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Open Coed NT Allstar L7</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Universitaire L2</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
         <is>
           <t>Universitaire L3</t>
         </is>

</xml_diff>

<commit_message>
fix: remove contact form
</commit_message>
<xml_diff>
--- a/public/docs/inscription-equipe.xlsx
+++ b/public/docs/inscription-equipe.xlsx
@@ -852,14 +852,14 @@
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>Ce document ne fait pas office de facture. Les tarifs affichés sur le site crown-cheerleading-events.fr font valeur de référence.</t>
+          <t>Ce document ne fait pas office de facture. Les tarifs affichés sur le site crown-cheerleading-events.org font valeur de référence.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="50" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>Un acompte de 30 % est requis à l'inscription. Toute annulation avant la fermeture des inscriptions donne droit à un remboursement de 70 %, les 30 % d'acompte restant acquis. Envoyez ce fichier à : contact@crown-cheerleading-events.org</t>
+          <t>Un acompte de 30 % est requis à l'inscription. Toute annulation avant la fermeture des inscriptions donne droit à un remboursement de 70 %, les 30 % d'acompte restant acquis. Le formulaire d'inscription pour l'envoi de ce fichier sera accessible à partir du 10 septembre 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: event at paris saclay
</commit_message>
<xml_diff>
--- a/public/docs/inscription-equipe.xlsx
+++ b/public/docs/inscription-equipe.xlsx
@@ -709,7 +709,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>4 avril 2027  ·  Dojo de Paris  ·  Un fichier par équipe</t>
+          <t>4 avril 2027  ·  Centre omnisports universitaire Carole Vergne  ·  Un fichier par équipe</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIF(Athlètes!E5:E200,"Masculin")</f>
+        <f>COUNTIF(Athlètes!E5:E39,"M")</f>
         <v/>
       </c>
     </row>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="C14" s="7">
-        <f>MAX(0,COUNTA(Accompagnateurs!B5:B24)-2)</f>
+        <f>MAX(0,COUNTA(Accompagnateurs!B5:B11)-2)</f>
         <v/>
       </c>
     </row>
@@ -828,11 +828,11 @@
         </is>
       </c>
       <c r="C17" s="9">
-        <f>IF(C8="Démo",37.5,IF(ISNUMBER(SEARCH("Novice",C8)),40,IF(OR(ISNUMBER(SEARCH("Allstar",C8)),ISNUMBER(SEARCH("Prep",C8)),ISNUMBER(SEARCH("Universitaire",C8))),50,IF(C8&lt;&gt;"","50",""))))</f>
+        <f>IF(C8="Démo",35,IF(ISNUMBER(SEARCH("Novice",C8)),35,IF(ISNUMBER(SEARCH("Allstar",C8)),45,IF(OR(ISNUMBER(SEARCH("Prep",C8)),ISNUMBER(SEARCH("Universitaire",C8))),40,IF(C8&lt;&gt;"","?","")))))</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>IF(C8="Démo","Démo : 37,50 €",IF(ISNUMBER(SEARCH("Novice",C8)),"Novice : 40 €",IF(OR(ISNUMBER(SEARCH("Allstar",C8)),ISNUMBER(SEARCH("Prep",C8)),ISNUMBER(SEARCH("Universitaire",C8))),"AllStar / Prep / Univ. : 50 €",IF(C8&lt;&gt;"","50 €","← sélectionnez une division"))))</f>
+        <f>IF(C8="Démo","Démo : 35 €",IF(ISNUMBER(SEARCH("Novice",C8)),"Novice : 35 €",IF(ISNUMBER(SEARCH("Allstar",C8)),"Allstar : 45 €",IF(OR(ISNUMBER(SEARCH("Prep",C8)),ISNUMBER(SEARCH("Universitaire",C8))),"Universitaire / Prep : 40 €",IF(C8&lt;&gt;"","? €","← sélectionnez une division")))))</f>
         <v/>
       </c>
     </row>
@@ -881,7 +881,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valeur invalide" error="Choisissez une division dans la liste" type="list">
-      <formula1>Listes!$A$1:$A$45</formula1>
+      <formula1>Listes!$A$1:$A$55</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1315,7 +1315,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Féminin,Masculin"</formula1>
+      <formula1>"F,M,Autre"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1352,7 +1352,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="29" t="inlineStr">
         <is>
-          <t>2 accompagnateurs par équipe sont inclus dans les frais d'inscription (lignes 1 et 2). Les suivants sont facturés 40 € chacun et comptabilisés automatiquement dans l'onglet Accueil.</t>
+          <t>2 accompagnateurs par équipe sont inclus dans les frais d'inscription (lignes 1 et 2). Les suivants sont facturés 40 € chacun et comptabilisés automatiquement dans l'onglet Accueil. Maximum 7 accompagnateurs.</t>
         </is>
       </c>
     </row>
@@ -1450,126 +1450,9 @@
       <c r="D11" s="20" t="n"/>
       <c r="E11" s="33" t="n"/>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="24" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="25" t="n"/>
-      <c r="C12" s="25" t="n"/>
-      <c r="D12" s="25" t="n"/>
-      <c r="E12" s="34" t="n"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="33" t="n"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="25" t="n"/>
-      <c r="C14" s="25" t="n"/>
-      <c r="D14" s="25" t="n"/>
-      <c r="E14" s="34" t="n"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="33" t="n"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="25" t="n"/>
-      <c r="C16" s="25" t="n"/>
-      <c r="D16" s="25" t="n"/>
-      <c r="E16" s="34" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="20" t="n"/>
-      <c r="C17" s="20" t="n"/>
-      <c r="D17" s="20" t="n"/>
-      <c r="E17" s="33" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="24" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="25" t="n"/>
-      <c r="C18" s="25" t="n"/>
-      <c r="D18" s="25" t="n"/>
-      <c r="E18" s="34" t="n"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="20" t="n"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="33" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="24" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="25" t="n"/>
-      <c r="C20" s="25" t="n"/>
-      <c r="D20" s="25" t="n"/>
-      <c r="E20" s="34" t="n"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="19" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="20" t="n"/>
-      <c r="C21" s="20" t="n"/>
-      <c r="D21" s="20" t="n"/>
-      <c r="E21" s="33" t="n"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="24" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="25" t="n"/>
-      <c r="C22" s="25" t="n"/>
-      <c r="D22" s="25" t="n"/>
-      <c r="E22" s="34" t="n"/>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="19" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="20" t="n"/>
-      <c r="C23" s="20" t="n"/>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="33" t="n"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="25" t="n"/>
-      <c r="C24" s="25" t="n"/>
-      <c r="D24" s="25" t="n"/>
-      <c r="E24" s="34" t="n"/>
-    </row>
-    <row r="25" ht="10" customHeight="1"/>
-    <row r="26" ht="50" customHeight="1">
-      <c r="A26" s="14" t="inlineStr">
+    <row r="12" ht="10" customHeight="1"/>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>RAPPEL RÈGLEMENT : Seuls les accompagnateurs et athlètes déclarés sont autorisés en salle d'échauffement et dans les vestiaires. Les accompagnateurs doivent arriver en même temps que leur équipe et se présenter à l'accueil pour récupérer leur bracelet.</t>
         </is>
@@ -1580,11 +1463,11 @@
   <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A13:E13"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5 E6 E7 E8 E9 E10 E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Entraîneur principal,Assistant entraîneur,Parent accompagnateur,Physio / Thérapeute,Photographe / Média,Autre"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1598,7 +1481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1625,7 +1508,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>U12 Prep L1</t>
+          <t>U12 Prep L1.1</t>
         </is>
       </c>
     </row>
@@ -1639,278 +1522,348 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>U16 Prep L1</t>
+          <t>U12 Prep L2.2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>U16 Prep L2.1</t>
+          <t>U16 Prep L1.1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>U18 Prep L1</t>
+          <t>U16 Prep L2.1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>U18 Prep L2.1</t>
+          <t>U16 Prep L2.2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Open Prep L1</t>
+          <t>U18 Prep L1.1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Open Prep L2.1</t>
+          <t>U18 Prep L2.1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>U12 Allstar L1</t>
+          <t>U18 Prep L2.2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>U12 Allstar L2</t>
+          <t>Open Prep L1.1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>U16 Allstar L1</t>
+          <t>Open Prep L2.1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>U16 Allstar L2</t>
+          <t>Open Prep L2.2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>U16 Allstar L3</t>
+          <t>U12 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>U18 Allstar L1</t>
+          <t>U12 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>U18 Allstar L2</t>
+          <t>U16 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>U18 Allstar L3</t>
+          <t>U16 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>U18 Allstar L4</t>
+          <t>U16 Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Open Allstar L1</t>
+          <t>U18 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Open Allstar L2</t>
+          <t>U18 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Open AG Allstar L3</t>
+          <t>U18 Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Open AG Allstar L4</t>
+          <t>U18 Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Open AG Allstar L5</t>
+          <t>U18 Allstar L4.2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Open AG Allstar L6</t>
+          <t>Open Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Open AG Allstar L7</t>
+          <t>Open Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L3</t>
+          <t>Open Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L4</t>
+          <t>Open AG Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L5</t>
+          <t>Open AG Allstar L4.2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L6</t>
+          <t>Open AG Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L7</t>
+          <t>Open AG Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Open NT Allstar L2</t>
+          <t>Open AG Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L3</t>
+          <t>Open Coed Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L4</t>
+          <t>Open Coed Allstar L4.2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L5</t>
+          <t>Open Coed Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L6</t>
+          <t>Open Coed Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L7</t>
+          <t>Open Coed Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L3</t>
+          <t>U16 NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L4</t>
+          <t>U16 NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L5</t>
+          <t>U18 NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L6</t>
+          <t>U18 NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L7</t>
+          <t>U18 NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Universitaire L2</t>
+          <t>Open NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
+        <is>
+          <t>Open NT Allstar L3</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Open AG NT Allstar L4</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Open AG NT Allstar L5</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Open AG NT Allstar L6</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Open AG NT Allstar L7</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Open Coed NT Allstar L4</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Open Coed NT Allstar L5</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Open Coed NT Allstar L6</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Open Coed NT Allstar L7</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Universitaire L2</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Universitaire L3</t>
         </is>

</xml_diff>

<commit_message>
fix: logo and categories
</commit_message>
<xml_diff>
--- a/public/docs/inscription-equipe.xlsx
+++ b/public/docs/inscription-equipe.xlsx
@@ -881,7 +881,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valeur invalide" error="Choisissez une division dans la liste" type="list">
-      <formula1>Listes!$A$1:$A$55</formula1>
+      <formula1>Listes!$A$1:$A$58</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1481,7 +1481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A55"/>
+  <dimension ref="A1:A58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1564,308 +1564,329 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Masters Prep L1.1</t>
+          <t>Open Prep L1.1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Masters Prep L2.1</t>
+          <t>Open Prep L2.1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Masters Prep L2.2</t>
+          <t>Open Prep L2.2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>U8 Allstar L1</t>
+          <t>Masters Prep L1.1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>U12 Allstar L1</t>
+          <t>Masters Prep L2.1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>U12 Allstar L2</t>
+          <t>Masters Prep L2.2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>U16 Allstar L1</t>
+          <t>U8 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>U16 Allstar L2</t>
+          <t>U12 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>U16 Allstar L3</t>
+          <t>U12 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>U18 Allstar L1</t>
+          <t>U16 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>U18 Allstar L2</t>
+          <t>U16 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>U18 Allstar L3</t>
+          <t>U16 Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>U18 Allstar L4</t>
+          <t>U18 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>U18 Allstar L4.2</t>
+          <t>U18 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Open Allstar L1</t>
+          <t>U18 Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Open Allstar L2</t>
+          <t>U18 Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Open Allstar L3</t>
+          <t>U18 Allstar L4.2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Open AG Allstar L4</t>
+          <t>Open Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Open AG Allstar L4.2</t>
+          <t>Open Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Open AG Allstar L5</t>
+          <t>Open Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Open AG Allstar L6</t>
+          <t>Open Allstar L4.2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Open AG Allstar L7</t>
+          <t>Open AG Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L4</t>
+          <t>Open AG Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L4.2</t>
+          <t>Open AG Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L5</t>
+          <t>Open AG Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L6</t>
+          <t>Open Coed Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L7</t>
+          <t>Open Coed Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>U16 NT Allstar L2</t>
+          <t>Open Coed Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>U16 NT Allstar L3</t>
+          <t>Open Coed Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>U18 NT Allstar L2</t>
+          <t>U16 NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>U18 NT Allstar L3</t>
+          <t>U16 NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>U18 NT Allstar L4</t>
+          <t>U18 NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Open NT Allstar L2</t>
+          <t>U18 NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Open NT Allstar L3</t>
+          <t>U18 NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L4</t>
+          <t>Open NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L5</t>
+          <t>Open NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L6</t>
+          <t>Open AG NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L7</t>
+          <t>Open AG NT Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L4</t>
+          <t>Open AG NT Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L5</t>
+          <t>Open AG NT Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L6</t>
+          <t>Open Coed NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L7</t>
+          <t>Open Coed NT Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Universitaire L2</t>
+          <t>Open Coed NT Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>Open Coed NT Allstar L7</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Universitaire L2</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>Universitaire L3</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Universitaire L4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add u16 level 4 division
</commit_message>
<xml_diff>
--- a/public/docs/inscription-equipe.xlsx
+++ b/public/docs/inscription-equipe.xlsx
@@ -709,7 +709,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>4 avril 2027  ·  Centre omnisports universitaire Carole Vergne  ·  Un fichier par équipe</t>
+          <t>4 avril 2027  ·  Centre Omnisports Universitaire Carole Vergne  ·  Un fichier par équipe</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A58"/>
+  <dimension ref="A1:A61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1648,243 +1648,264 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>U18 Allstar L1</t>
+          <t>U16 Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>U18 Allstar L2</t>
+          <t>U16 Allstar L4.2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>U18 Allstar L3</t>
+          <t>U18 Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>U18 Allstar L4</t>
+          <t>U18 Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>U18 Allstar L4.2</t>
+          <t>U18 Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Open Allstar L1</t>
+          <t>U18 Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Open Allstar L2</t>
+          <t>U18 Allstar L4.2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Open Allstar L3</t>
+          <t>Open Allstar L1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Open Allstar L4.2</t>
+          <t>Open Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Open AG Allstar L4</t>
+          <t>Open Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Open AG Allstar L5</t>
+          <t>Open Allstar L4.2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Open AG Allstar L6</t>
+          <t>Open AG Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Open AG Allstar L7</t>
+          <t>Open AG Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L4</t>
+          <t>Open AG Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L5</t>
+          <t>Open AG Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L6</t>
+          <t>Open Coed Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Open Coed Allstar L7</t>
+          <t>Open Coed Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>U16 NT Allstar L2</t>
+          <t>Open Coed Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>U16 NT Allstar L3</t>
+          <t>Open Coed Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>U18 NT Allstar L2</t>
+          <t>U16 NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>U18 NT Allstar L3</t>
+          <t>U16 NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>U18 NT Allstar L4</t>
+          <t>U16 NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Open NT Allstar L2</t>
+          <t>U18 NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Open NT Allstar L3</t>
+          <t>U18 NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L4</t>
+          <t>U18 NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L5</t>
+          <t>Open NT Allstar L2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L6</t>
+          <t>Open NT Allstar L3</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Open AG NT Allstar L7</t>
+          <t>Open AG NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L4</t>
+          <t>Open AG NT Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L5</t>
+          <t>Open AG NT Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L6</t>
+          <t>Open AG NT Allstar L7</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Open Coed NT Allstar L7</t>
+          <t>Open Coed NT Allstar L4</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Universitaire L2</t>
+          <t>Open Coed NT Allstar L5</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Universitaire L3</t>
+          <t>Open Coed NT Allstar L6</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
+        <is>
+          <t>Open Coed NT Allstar L7</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Universitaire L2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Universitaire L3</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>Universitaire L4</t>
         </is>

</xml_diff>

<commit_message>
feat: add warning excel
</commit_message>
<xml_diff>
--- a/public/docs/inscription-equipe.xlsx
+++ b/public/docs/inscription-equipe.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +57,12 @@
       <name val="Calibri"/>
       <color rgb="001A1A1A"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -120,7 +126,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -150,6 +156,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B00000"/>
       </patternFill>
     </fill>
   </fills>
@@ -206,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -227,41 +238,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -272,7 +286,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -280,7 +294,7 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -291,7 +305,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -299,17 +313,17 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -687,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -766,98 +780,105 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>⚠ Les calculs ci-dessous sont automatiques et se mettent à jour en remplissant la feuille. Ne pas modifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Nombre total d'athlètes</t>
         </is>
       </c>
-      <c r="C11" s="7">
+      <c r="C12" s="8">
         <f>COUNTA(Athlètes!B5:B39)</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Dont athlètes masculins</t>
         </is>
       </c>
-      <c r="C12" s="7">
+      <c r="C13" s="8">
         <f>COUNTIF(Athlètes!E5:E39,"M")</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Accompagnateurs inclus (2/équipe)</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>Accompagnateurs inclus (2/équipe)</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
           <t>Accompagnateurs supplémentaires</t>
         </is>
       </c>
-      <c r="C14" s="7">
+      <c r="C15" s="8">
         <f>MAX(0,COUNTA(Accompagnateurs!B5:B11)-2)</f>
         <v/>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Coût accompagnateurs suppl. (€)</t>
         </is>
       </c>
-      <c r="C15" s="7">
-        <f>C14*40</f>
+      <c r="C16" s="8">
+        <f>C15*40</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="10" customHeight="1"/>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="17" ht="10" customHeight="1"/>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">  Prix par athlète (€)</t>
         </is>
       </c>
-      <c r="C17" s="9">
+      <c r="C18" s="10">
         <f>IF(C8="Démo",35,IF(ISNUMBER(SEARCH("Allstar",C8)),40,IF(OR(ISNUMBER(SEARCH("Prep",C8)),ISNUMBER(SEARCH("Universitaire",C8))),37.5,IF(C8&lt;&gt;"","?",""))))</f>
         <v/>
       </c>
-      <c r="D17" s="10">
+      <c r="D18" s="11">
         <f>IF(C8="Démo","Démo : 35 €",IF(ISNUMBER(SEARCH("Allstar",C8)),"Allstar : 40 €",IF(OR(ISNUMBER(SEARCH("Prep",C8)),ISNUMBER(SEARCH("Universitaire",C8))),"Universitaire / Prep : 37,50 €",IF(C8&lt;&gt;"","? €","← sélectionnez une division"))))</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="10" customHeight="1"/>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="19" ht="10" customHeight="1"/>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  TOTAL ESTIMÉ (athlètes + accomp. suppl.)</t>
         </is>
       </c>
-      <c r="C19" s="12">
-        <f>C11*C17+C15</f>
+      <c r="C20" s="13">
+        <f>C12*C18+C16</f>
         <v/>
       </c>
     </row>
-    <row r="20" ht="10" customHeight="1"/>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="21" ht="10" customHeight="1"/>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Ce document ne fait pas office de facture. Les tarifs affichés sur le site crown-cheerleading-events.fr font valeur de référence.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="50" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Un acompte de 30 % est requis à l'inscription. Toute annulation avant la fermeture des inscriptions donne droit à un remboursement de 70 %, les 30 % d'acompte restant acquis. Le formulaire d'inscription pour l'envoi de ce fichier sera accessible à partir du 10 septembre 2026.</t>
         </is>
@@ -865,19 +886,20 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <mergeCells count="12">
+  <mergeCells count="13">
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="A20:B20"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="D17:G17"/>
     <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
     <mergeCell ref="C8:G8"/>
+    <mergeCell ref="A11:G11"/>
     <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valeur invalide" error="Choisissez une division dans la liste" type="list">
@@ -907,404 +929,404 @@
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>LISTE DES ATHLÈTES</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="16" t="n"/>
+      <c r="A2" s="17" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>← Équipe : voir feuille "Accueil"</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Nom</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Prénom</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>Date de naissance
 (JJ/MM/AAAA)</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>Sexe</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="19" t="inlineStr">
         <is>
           <t>Remarque</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="19" t="n">
+      <c r="A5" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="20" t="n"/>
-      <c r="C5" s="20" t="n"/>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="22" t="n"/>
-      <c r="F5" s="23" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="23" t="n"/>
+      <c r="F5" s="24" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="24" t="n">
+      <c r="A6" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="25" t="n"/>
-      <c r="C6" s="25" t="n"/>
-      <c r="D6" s="26" t="n"/>
-      <c r="E6" s="27" t="n"/>
-      <c r="F6" s="28" t="n"/>
+      <c r="B6" s="26" t="n"/>
+      <c r="C6" s="26" t="n"/>
+      <c r="D6" s="27" t="n"/>
+      <c r="E6" s="28" t="n"/>
+      <c r="F6" s="29" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="20" t="n"/>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="22" t="n"/>
-      <c r="F7" s="23" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="23" t="n"/>
+      <c r="F7" s="24" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="24" t="n">
+      <c r="A8" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="25" t="n"/>
-      <c r="C8" s="25" t="n"/>
-      <c r="D8" s="26" t="n"/>
-      <c r="E8" s="27" t="n"/>
-      <c r="F8" s="28" t="n"/>
+      <c r="B8" s="26" t="n"/>
+      <c r="C8" s="26" t="n"/>
+      <c r="D8" s="27" t="n"/>
+      <c r="E8" s="28" t="n"/>
+      <c r="F8" s="29" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="20" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="22" t="n"/>
-      <c r="F9" s="23" t="n"/>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="23" t="n"/>
+      <c r="F9" s="24" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="24" t="n">
+      <c r="A10" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="25" t="n"/>
-      <c r="C10" s="25" t="n"/>
-      <c r="D10" s="26" t="n"/>
-      <c r="E10" s="27" t="n"/>
-      <c r="F10" s="28" t="n"/>
+      <c r="B10" s="26" t="n"/>
+      <c r="C10" s="26" t="n"/>
+      <c r="D10" s="27" t="n"/>
+      <c r="E10" s="28" t="n"/>
+      <c r="F10" s="29" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="19" t="n">
+      <c r="A11" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="20" t="n"/>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="22" t="n"/>
-      <c r="F11" s="23" t="n"/>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="23" t="n"/>
+      <c r="F11" s="24" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="24" t="n">
+      <c r="A12" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="25" t="n"/>
-      <c r="C12" s="25" t="n"/>
-      <c r="D12" s="26" t="n"/>
-      <c r="E12" s="27" t="n"/>
-      <c r="F12" s="28" t="n"/>
+      <c r="B12" s="26" t="n"/>
+      <c r="C12" s="26" t="n"/>
+      <c r="D12" s="27" t="n"/>
+      <c r="E12" s="28" t="n"/>
+      <c r="F12" s="29" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="19" t="n">
+      <c r="A13" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="23" t="n"/>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="22" t="n"/>
+      <c r="E13" s="23" t="n"/>
+      <c r="F13" s="24" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="24" t="n">
+      <c r="A14" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="25" t="n"/>
-      <c r="C14" s="25" t="n"/>
-      <c r="D14" s="26" t="n"/>
-      <c r="E14" s="27" t="n"/>
-      <c r="F14" s="28" t="n"/>
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="27" t="n"/>
+      <c r="E14" s="28" t="n"/>
+      <c r="F14" s="29" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="19" t="n">
+      <c r="A15" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="21" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="23" t="n"/>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="22" t="n"/>
+      <c r="E15" s="23" t="n"/>
+      <c r="F15" s="24" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="24" t="n">
+      <c r="A16" s="25" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="25" t="n"/>
-      <c r="C16" s="25" t="n"/>
-      <c r="D16" s="26" t="n"/>
-      <c r="E16" s="27" t="n"/>
-      <c r="F16" s="28" t="n"/>
+      <c r="B16" s="26" t="n"/>
+      <c r="C16" s="26" t="n"/>
+      <c r="D16" s="27" t="n"/>
+      <c r="E16" s="28" t="n"/>
+      <c r="F16" s="29" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="19" t="n">
+      <c r="A17" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="20" t="n"/>
-      <c r="C17" s="20" t="n"/>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="22" t="n"/>
-      <c r="F17" s="23" t="n"/>
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="22" t="n"/>
+      <c r="E17" s="23" t="n"/>
+      <c r="F17" s="24" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="24" t="n">
+      <c r="A18" s="25" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="25" t="n"/>
-      <c r="C18" s="25" t="n"/>
-      <c r="D18" s="26" t="n"/>
-      <c r="E18" s="27" t="n"/>
-      <c r="F18" s="28" t="n"/>
+      <c r="B18" s="26" t="n"/>
+      <c r="C18" s="26" t="n"/>
+      <c r="D18" s="27" t="n"/>
+      <c r="E18" s="28" t="n"/>
+      <c r="F18" s="29" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="19" t="n">
+      <c r="A19" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="20" t="n"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="21" t="n"/>
-      <c r="E19" s="22" t="n"/>
-      <c r="F19" s="23" t="n"/>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="22" t="n"/>
+      <c r="E19" s="23" t="n"/>
+      <c r="F19" s="24" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="24" t="n">
+      <c r="A20" s="25" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="25" t="n"/>
-      <c r="C20" s="25" t="n"/>
-      <c r="D20" s="26" t="n"/>
-      <c r="E20" s="27" t="n"/>
-      <c r="F20" s="28" t="n"/>
+      <c r="B20" s="26" t="n"/>
+      <c r="C20" s="26" t="n"/>
+      <c r="D20" s="27" t="n"/>
+      <c r="E20" s="28" t="n"/>
+      <c r="F20" s="29" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="19" t="n">
+      <c r="A21" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="20" t="n"/>
-      <c r="C21" s="20" t="n"/>
-      <c r="D21" s="21" t="n"/>
-      <c r="E21" s="22" t="n"/>
-      <c r="F21" s="23" t="n"/>
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="21" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="23" t="n"/>
+      <c r="F21" s="24" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="24" t="n">
+      <c r="A22" s="25" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="25" t="n"/>
-      <c r="C22" s="25" t="n"/>
-      <c r="D22" s="26" t="n"/>
-      <c r="E22" s="27" t="n"/>
-      <c r="F22" s="28" t="n"/>
+      <c r="B22" s="26" t="n"/>
+      <c r="C22" s="26" t="n"/>
+      <c r="D22" s="27" t="n"/>
+      <c r="E22" s="28" t="n"/>
+      <c r="F22" s="29" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="19" t="n">
+      <c r="A23" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="20" t="n"/>
-      <c r="C23" s="20" t="n"/>
-      <c r="D23" s="21" t="n"/>
-      <c r="E23" s="22" t="n"/>
-      <c r="F23" s="23" t="n"/>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="24" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="24" t="n">
+      <c r="A24" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="25" t="n"/>
-      <c r="C24" s="25" t="n"/>
-      <c r="D24" s="26" t="n"/>
-      <c r="E24" s="27" t="n"/>
-      <c r="F24" s="28" t="n"/>
+      <c r="B24" s="26" t="n"/>
+      <c r="C24" s="26" t="n"/>
+      <c r="D24" s="27" t="n"/>
+      <c r="E24" s="28" t="n"/>
+      <c r="F24" s="29" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="19" t="n">
+      <c r="A25" s="20" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="20" t="n"/>
-      <c r="C25" s="20" t="n"/>
-      <c r="D25" s="21" t="n"/>
-      <c r="E25" s="22" t="n"/>
-      <c r="F25" s="23" t="n"/>
+      <c r="B25" s="21" t="n"/>
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="23" t="n"/>
+      <c r="F25" s="24" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="24" t="n">
+      <c r="A26" s="25" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="25" t="n"/>
-      <c r="C26" s="25" t="n"/>
-      <c r="D26" s="26" t="n"/>
-      <c r="E26" s="27" t="n"/>
-      <c r="F26" s="28" t="n"/>
+      <c r="B26" s="26" t="n"/>
+      <c r="C26" s="26" t="n"/>
+      <c r="D26" s="27" t="n"/>
+      <c r="E26" s="28" t="n"/>
+      <c r="F26" s="29" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="19" t="n">
+      <c r="A27" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="20" t="n"/>
-      <c r="C27" s="20" t="n"/>
-      <c r="D27" s="21" t="n"/>
-      <c r="E27" s="22" t="n"/>
-      <c r="F27" s="23" t="n"/>
+      <c r="B27" s="21" t="n"/>
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="23" t="n"/>
+      <c r="F27" s="24" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="24" t="n">
+      <c r="A28" s="25" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="25" t="n"/>
-      <c r="C28" s="25" t="n"/>
-      <c r="D28" s="26" t="n"/>
-      <c r="E28" s="27" t="n"/>
-      <c r="F28" s="28" t="n"/>
+      <c r="B28" s="26" t="n"/>
+      <c r="C28" s="26" t="n"/>
+      <c r="D28" s="27" t="n"/>
+      <c r="E28" s="28" t="n"/>
+      <c r="F28" s="29" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="19" t="n">
+      <c r="A29" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="20" t="n"/>
-      <c r="C29" s="20" t="n"/>
-      <c r="D29" s="21" t="n"/>
-      <c r="E29" s="22" t="n"/>
-      <c r="F29" s="23" t="n"/>
+      <c r="B29" s="21" t="n"/>
+      <c r="C29" s="21" t="n"/>
+      <c r="D29" s="22" t="n"/>
+      <c r="E29" s="23" t="n"/>
+      <c r="F29" s="24" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="24" t="n">
+      <c r="A30" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="26" t="n"/>
-      <c r="E30" s="27" t="n"/>
-      <c r="F30" s="28" t="n"/>
+      <c r="B30" s="26" t="n"/>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="28" t="n"/>
+      <c r="F30" s="29" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="19" t="n">
+      <c r="A31" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="20" t="n"/>
-      <c r="C31" s="20" t="n"/>
-      <c r="D31" s="21" t="n"/>
-      <c r="E31" s="22" t="n"/>
-      <c r="F31" s="23" t="n"/>
+      <c r="B31" s="21" t="n"/>
+      <c r="C31" s="21" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="23" t="n"/>
+      <c r="F31" s="24" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="24" t="n">
+      <c r="A32" s="25" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="25" t="n"/>
-      <c r="C32" s="25" t="n"/>
-      <c r="D32" s="26" t="n"/>
-      <c r="E32" s="27" t="n"/>
-      <c r="F32" s="28" t="n"/>
+      <c r="B32" s="26" t="n"/>
+      <c r="C32" s="26" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="28" t="n"/>
+      <c r="F32" s="29" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="19" t="n">
+      <c r="A33" s="20" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="20" t="n"/>
-      <c r="C33" s="20" t="n"/>
-      <c r="D33" s="21" t="n"/>
-      <c r="E33" s="22" t="n"/>
-      <c r="F33" s="23" t="n"/>
+      <c r="B33" s="21" t="n"/>
+      <c r="C33" s="21" t="n"/>
+      <c r="D33" s="22" t="n"/>
+      <c r="E33" s="23" t="n"/>
+      <c r="F33" s="24" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="24" t="n">
+      <c r="A34" s="25" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="25" t="n"/>
-      <c r="C34" s="25" t="n"/>
-      <c r="D34" s="26" t="n"/>
-      <c r="E34" s="27" t="n"/>
-      <c r="F34" s="28" t="n"/>
+      <c r="B34" s="26" t="n"/>
+      <c r="C34" s="26" t="n"/>
+      <c r="D34" s="27" t="n"/>
+      <c r="E34" s="28" t="n"/>
+      <c r="F34" s="29" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="19" t="n">
+      <c r="A35" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="20" t="n"/>
-      <c r="C35" s="20" t="n"/>
-      <c r="D35" s="21" t="n"/>
-      <c r="E35" s="22" t="n"/>
-      <c r="F35" s="23" t="n"/>
+      <c r="B35" s="21" t="n"/>
+      <c r="C35" s="21" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="23" t="n"/>
+      <c r="F35" s="24" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="24" t="n">
+      <c r="A36" s="25" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="25" t="n"/>
-      <c r="C36" s="25" t="n"/>
-      <c r="D36" s="26" t="n"/>
-      <c r="E36" s="27" t="n"/>
-      <c r="F36" s="28" t="n"/>
+      <c r="B36" s="26" t="n"/>
+      <c r="C36" s="26" t="n"/>
+      <c r="D36" s="27" t="n"/>
+      <c r="E36" s="28" t="n"/>
+      <c r="F36" s="29" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="19" t="n">
+      <c r="A37" s="20" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="20" t="n"/>
-      <c r="C37" s="20" t="n"/>
-      <c r="D37" s="21" t="n"/>
-      <c r="E37" s="22" t="n"/>
-      <c r="F37" s="23" t="n"/>
+      <c r="B37" s="21" t="n"/>
+      <c r="C37" s="21" t="n"/>
+      <c r="D37" s="22" t="n"/>
+      <c r="E37" s="23" t="n"/>
+      <c r="F37" s="24" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="24" t="n">
+      <c r="A38" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="25" t="n"/>
-      <c r="C38" s="25" t="n"/>
-      <c r="D38" s="26" t="n"/>
-      <c r="E38" s="27" t="n"/>
-      <c r="F38" s="28" t="n"/>
+      <c r="B38" s="26" t="n"/>
+      <c r="C38" s="26" t="n"/>
+      <c r="D38" s="27" t="n"/>
+      <c r="E38" s="28" t="n"/>
+      <c r="F38" s="29" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="19" t="n">
+      <c r="A39" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="20" t="n"/>
-      <c r="C39" s="20" t="n"/>
-      <c r="D39" s="21" t="n"/>
-      <c r="E39" s="22" t="n"/>
-      <c r="F39" s="23" t="n"/>
+      <c r="B39" s="21" t="n"/>
+      <c r="C39" s="21" t="n"/>
+      <c r="D39" s="22" t="n"/>
+      <c r="E39" s="23" t="n"/>
+      <c r="F39" s="24" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
@@ -1340,119 +1362,119 @@
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>ENTRAÎNEURS &amp; ACCOMPAGNATEURS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="16" t="n"/>
+      <c r="A2" s="17" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="29" t="inlineStr">
+      <c r="A3" s="30" t="inlineStr">
         <is>
           <t>2 accompagnateurs par équipe sont inclus dans les frais d'inscription (lignes 1 et 2). Les suivants sont facturés 40 € chacun et comptabilisés automatiquement dans l'onglet Accueil. Maximum 7 accompagnateurs.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Nom</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Prénom</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>Email (obligatoire pour entraîneur)</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>Rôle</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>1 ✓</t>
         </is>
       </c>
-      <c r="B5" s="31" t="n"/>
-      <c r="C5" s="31" t="n"/>
-      <c r="D5" s="31" t="n"/>
-      <c r="E5" s="32" t="n"/>
+      <c r="B5" s="32" t="n"/>
+      <c r="C5" s="32" t="n"/>
+      <c r="D5" s="32" t="n"/>
+      <c r="E5" s="33" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>2 ✓</t>
         </is>
       </c>
-      <c r="B6" s="31" t="n"/>
-      <c r="C6" s="31" t="n"/>
-      <c r="D6" s="31" t="n"/>
-      <c r="E6" s="32" t="n"/>
+      <c r="B6" s="32" t="n"/>
+      <c r="C6" s="32" t="n"/>
+      <c r="D6" s="32" t="n"/>
+      <c r="E6" s="33" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="20" t="n"/>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="33" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="34" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="24" t="n">
+      <c r="A8" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="25" t="n"/>
-      <c r="C8" s="25" t="n"/>
-      <c r="D8" s="25" t="n"/>
-      <c r="E8" s="34" t="n"/>
+      <c r="B8" s="26" t="n"/>
+      <c r="C8" s="26" t="n"/>
+      <c r="D8" s="26" t="n"/>
+      <c r="E8" s="35" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="20" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="33" t="n"/>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="34" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="24" t="n">
+      <c r="A10" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="25" t="n"/>
-      <c r="C10" s="25" t="n"/>
-      <c r="D10" s="25" t="n"/>
-      <c r="E10" s="34" t="n"/>
+      <c r="B10" s="26" t="n"/>
+      <c r="C10" s="26" t="n"/>
+      <c r="D10" s="26" t="n"/>
+      <c r="E10" s="35" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="19" t="n">
+      <c r="A11" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="20" t="n"/>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="33" t="n"/>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="34" t="n"/>
     </row>
     <row r="12" ht="10" customHeight="1"/>
     <row r="13" ht="50" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>RAPPEL RÈGLEMENT : Seuls les accompagnateurs et athlètes déclarés sont autorisés en salle d'échauffement et dans les vestiaires. Les accompagnateurs doivent arriver en même temps que leur équipe et se présenter à l'accueil pour récupérer leur bracelet.</t>
         </is>

</xml_diff>

<commit_message>
feat: add new summary page in excel
</commit_message>
<xml_diff>
--- a/public/docs/inscription-equipe.xlsx
+++ b/public/docs/inscription-equipe.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Accueil" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Athlètes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Accompagnateurs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Listes" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="Résumé" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Listes" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00 €"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -61,6 +63,39 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00D4AF37"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00555555"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00D4AF37"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00D4AF37"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
@@ -68,11 +103,6 @@
       <name val="Calibri"/>
       <color rgb="00D4AF37"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00555555"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -94,34 +124,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00D4AF37"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="001A1A1A"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00555555"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00D4AF37"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00D4AF37"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="001A1A1A"/>
       <sz val="9"/>
     </font>
@@ -187,14 +189,6 @@
       <diagonal/>
     </border>
     <border>
-      <top style="medium">
-        <color rgb="00D4AF37"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="00D4AF37"/>
-      </bottom>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="00A0820A"/>
       </left>
@@ -213,11 +207,19 @@
         <color rgb="00F0F0F0"/>
       </bottom>
     </border>
+    <border>
+      <top style="medium">
+        <color rgb="00D4AF37"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00D4AF37"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -238,55 +240,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -294,18 +269,18 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -313,17 +288,17 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -334,6 +309,36 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -701,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -773,133 +778,15 @@
       <c r="G8" s="6" t="n"/>
     </row>
     <row r="9" ht="10" customHeight="1"/>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  RÉSUMÉ &amp; CALCUL DES FRAIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>⚠ Les calculs ci-dessous sont automatiques et se mettent à jour en remplissant la feuille. Ne pas modifier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Nombre total d'athlètes</t>
-        </is>
-      </c>
-      <c r="C12" s="8">
-        <f>COUNTA(Athlètes!B5:B39)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Dont athlètes masculins</t>
-        </is>
-      </c>
-      <c r="C13" s="8">
-        <f>COUNTIF(Athlètes!E5:E39,"M")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Accompagnateurs inclus (2/équipe)</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Accompagnateurs supplémentaires</t>
-        </is>
-      </c>
-      <c r="C15" s="8">
-        <f>MAX(0,COUNTA(Accompagnateurs!B5:B11)-2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Coût accompagnateurs suppl. (€)</t>
-        </is>
-      </c>
-      <c r="C16" s="8">
-        <f>C15*40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="10" customHeight="1"/>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Prix par athlète (€)</t>
-        </is>
-      </c>
-      <c r="C18" s="10">
-        <f>IF(C8="Démo",35,IF(ISNUMBER(SEARCH("Allstar",C8)),40,IF(OR(ISNUMBER(SEARCH("Prep",C8)),ISNUMBER(SEARCH("Universitaire",C8))),37.5,IF(C8&lt;&gt;"","?",""))))</f>
-        <v/>
-      </c>
-      <c r="D18" s="11">
-        <f>IF(C8="Démo","Démo : 35 €",IF(ISNUMBER(SEARCH("Allstar",C8)),"Allstar : 40 €",IF(OR(ISNUMBER(SEARCH("Prep",C8)),ISNUMBER(SEARCH("Universitaire",C8))),"Universitaire / Prep : 37,50 €",IF(C8&lt;&gt;"","? €","← sélectionnez une division"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="10" customHeight="1"/>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  TOTAL ESTIMÉ (athlètes + accomp. suppl.)</t>
-        </is>
-      </c>
-      <c r="C20" s="13">
-        <f>C12*C18+C16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="10" customHeight="1"/>
-    <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>Ce document ne fait pas office de facture. Les tarifs affichés sur le site crown-cheerleading-events.fr font valeur de référence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="50" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>Un acompte de 30 % est requis à l'inscription. Toute annulation avant la fermeture des inscriptions donne droit à un remboursement de 70 %, les 30 % d'acompte restant acquis. Le formulaire d'inscription pour l'envoi de ce fichier sera accessible à partir du 10 septembre 2026.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <mergeCells count="13">
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="A20:B20"/>
+  <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A18:B18"/>
     <mergeCell ref="C8:G8"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valeur invalide" error="Choisissez une division dans la liste" type="list">
@@ -929,404 +816,404 @@
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>LISTE DES ATHLÈTES</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="17" t="n"/>
+      <c r="A2" s="8" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>← Équipe : voir feuille "Accueil"</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Nom</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Prénom</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Date de naissance
 (JJ/MM/AAAA)</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Sexe</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Remarque</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="20" t="n">
+      <c r="A5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="21" t="n"/>
-      <c r="C5" s="21" t="n"/>
-      <c r="D5" s="22" t="n"/>
-      <c r="E5" s="23" t="n"/>
-      <c r="F5" s="24" t="n"/>
+      <c r="B5" s="12" t="n"/>
+      <c r="C5" s="12" t="n"/>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="14" t="n"/>
+      <c r="F5" s="15" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="25" t="n">
+      <c r="A6" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="26" t="n"/>
-      <c r="C6" s="26" t="n"/>
-      <c r="D6" s="27" t="n"/>
-      <c r="E6" s="28" t="n"/>
-      <c r="F6" s="29" t="n"/>
+      <c r="B6" s="17" t="n"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="20" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="20" t="n">
+      <c r="A7" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="21" t="n"/>
-      <c r="C7" s="21" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="23" t="n"/>
-      <c r="F7" s="24" t="n"/>
+      <c r="B7" s="12" t="n"/>
+      <c r="C7" s="12" t="n"/>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="14" t="n"/>
+      <c r="F7" s="15" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="25" t="n">
+      <c r="A8" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="26" t="n"/>
-      <c r="C8" s="26" t="n"/>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="28" t="n"/>
-      <c r="F8" s="29" t="n"/>
+      <c r="B8" s="17" t="n"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="20" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="20" t="n">
+      <c r="A9" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="21" t="n"/>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="22" t="n"/>
-      <c r="E9" s="23" t="n"/>
-      <c r="F9" s="24" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="14" t="n"/>
+      <c r="F9" s="15" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="25" t="n">
+      <c r="A10" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="26" t="n"/>
-      <c r="D10" s="27" t="n"/>
-      <c r="E10" s="28" t="n"/>
-      <c r="F10" s="29" t="n"/>
+      <c r="B10" s="17" t="n"/>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="20" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="20" t="n">
+      <c r="A11" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="21" t="n"/>
-      <c r="C11" s="21" t="n"/>
-      <c r="D11" s="22" t="n"/>
-      <c r="E11" s="23" t="n"/>
-      <c r="F11" s="24" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="15" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="25" t="n">
+      <c r="A12" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="26" t="n"/>
-      <c r="C12" s="26" t="n"/>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="28" t="n"/>
-      <c r="F12" s="29" t="n"/>
+      <c r="B12" s="17" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="20" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="20" t="n">
+      <c r="A13" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="21" t="n"/>
-      <c r="C13" s="21" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="23" t="n"/>
-      <c r="F13" s="24" t="n"/>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="15" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="25" t="n">
+      <c r="A14" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="26" t="n"/>
-      <c r="C14" s="26" t="n"/>
-      <c r="D14" s="27" t="n"/>
-      <c r="E14" s="28" t="n"/>
-      <c r="F14" s="29" t="n"/>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="18" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="20" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="20" t="n">
+      <c r="A15" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="21" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="23" t="n"/>
-      <c r="F15" s="24" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="14" t="n"/>
+      <c r="F15" s="15" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="25" t="n">
+      <c r="A16" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="26" t="n"/>
-      <c r="C16" s="26" t="n"/>
-      <c r="D16" s="27" t="n"/>
-      <c r="E16" s="28" t="n"/>
-      <c r="F16" s="29" t="n"/>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="20" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="20" t="n">
+      <c r="A17" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="21" t="n"/>
-      <c r="C17" s="21" t="n"/>
-      <c r="D17" s="22" t="n"/>
-      <c r="E17" s="23" t="n"/>
-      <c r="F17" s="24" t="n"/>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="14" t="n"/>
+      <c r="F17" s="15" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="25" t="n">
+      <c r="A18" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="26" t="n"/>
-      <c r="C18" s="26" t="n"/>
-      <c r="D18" s="27" t="n"/>
-      <c r="E18" s="28" t="n"/>
-      <c r="F18" s="29" t="n"/>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="18" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="20" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="20" t="n">
+      <c r="A19" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="21" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="22" t="n"/>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="24" t="n"/>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="14" t="n"/>
+      <c r="F19" s="15" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="25" t="n">
+      <c r="A20" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="26" t="n"/>
-      <c r="C20" s="26" t="n"/>
-      <c r="D20" s="27" t="n"/>
-      <c r="E20" s="28" t="n"/>
-      <c r="F20" s="29" t="n"/>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="18" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="20" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="20" t="n">
+      <c r="A21" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="21" t="n"/>
-      <c r="C21" s="21" t="n"/>
-      <c r="D21" s="22" t="n"/>
-      <c r="E21" s="23" t="n"/>
-      <c r="F21" s="24" t="n"/>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="13" t="n"/>
+      <c r="E21" s="14" t="n"/>
+      <c r="F21" s="15" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="25" t="n">
+      <c r="A22" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="26" t="n"/>
-      <c r="C22" s="26" t="n"/>
-      <c r="D22" s="27" t="n"/>
-      <c r="E22" s="28" t="n"/>
-      <c r="F22" s="29" t="n"/>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="19" t="n"/>
+      <c r="F22" s="20" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="20" t="n">
+      <c r="A23" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="21" t="n"/>
-      <c r="C23" s="21" t="n"/>
-      <c r="D23" s="22" t="n"/>
-      <c r="E23" s="23" t="n"/>
-      <c r="F23" s="24" t="n"/>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="15" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="25" t="n">
+      <c r="A24" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="26" t="n"/>
-      <c r="C24" s="26" t="n"/>
-      <c r="D24" s="27" t="n"/>
-      <c r="E24" s="28" t="n"/>
-      <c r="F24" s="29" t="n"/>
+      <c r="B24" s="17" t="n"/>
+      <c r="C24" s="17" t="n"/>
+      <c r="D24" s="18" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="20" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="20" t="n">
+      <c r="A25" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="21" t="n"/>
-      <c r="C25" s="21" t="n"/>
-      <c r="D25" s="22" t="n"/>
-      <c r="E25" s="23" t="n"/>
-      <c r="F25" s="24" t="n"/>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="15" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="25" t="n">
+      <c r="A26" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="26" t="n"/>
-      <c r="C26" s="26" t="n"/>
-      <c r="D26" s="27" t="n"/>
-      <c r="E26" s="28" t="n"/>
-      <c r="F26" s="29" t="n"/>
+      <c r="B26" s="17" t="n"/>
+      <c r="C26" s="17" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="20" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="20" t="n">
+      <c r="A27" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="21" t="n"/>
-      <c r="C27" s="21" t="n"/>
-      <c r="D27" s="22" t="n"/>
-      <c r="E27" s="23" t="n"/>
-      <c r="F27" s="24" t="n"/>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="14" t="n"/>
+      <c r="F27" s="15" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="25" t="n">
+      <c r="A28" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="26" t="n"/>
-      <c r="C28" s="26" t="n"/>
-      <c r="D28" s="27" t="n"/>
-      <c r="E28" s="28" t="n"/>
-      <c r="F28" s="29" t="n"/>
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="17" t="n"/>
+      <c r="D28" s="18" t="n"/>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="20" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="20" t="n">
+      <c r="A29" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="21" t="n"/>
-      <c r="C29" s="21" t="n"/>
-      <c r="D29" s="22" t="n"/>
-      <c r="E29" s="23" t="n"/>
-      <c r="F29" s="24" t="n"/>
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="15" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="25" t="n">
+      <c r="A30" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="26" t="n"/>
-      <c r="C30" s="26" t="n"/>
-      <c r="D30" s="27" t="n"/>
-      <c r="E30" s="28" t="n"/>
-      <c r="F30" s="29" t="n"/>
+      <c r="B30" s="17" t="n"/>
+      <c r="C30" s="17" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="20" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="20" t="n">
+      <c r="A31" s="11" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="21" t="n"/>
-      <c r="C31" s="21" t="n"/>
-      <c r="D31" s="22" t="n"/>
-      <c r="E31" s="23" t="n"/>
-      <c r="F31" s="24" t="n"/>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="13" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="15" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="25" t="n">
+      <c r="A32" s="16" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="26" t="n"/>
-      <c r="C32" s="26" t="n"/>
-      <c r="D32" s="27" t="n"/>
-      <c r="E32" s="28" t="n"/>
-      <c r="F32" s="29" t="n"/>
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="17" t="n"/>
+      <c r="D32" s="18" t="n"/>
+      <c r="E32" s="19" t="n"/>
+      <c r="F32" s="20" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="20" t="n">
+      <c r="A33" s="11" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="21" t="n"/>
-      <c r="C33" s="21" t="n"/>
-      <c r="D33" s="22" t="n"/>
-      <c r="E33" s="23" t="n"/>
-      <c r="F33" s="24" t="n"/>
+      <c r="B33" s="12" t="n"/>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="13" t="n"/>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="15" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="25" t="n">
+      <c r="A34" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="26" t="n"/>
-      <c r="C34" s="26" t="n"/>
-      <c r="D34" s="27" t="n"/>
-      <c r="E34" s="28" t="n"/>
-      <c r="F34" s="29" t="n"/>
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="17" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="20" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="20" t="n">
+      <c r="A35" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="21" t="n"/>
-      <c r="C35" s="21" t="n"/>
-      <c r="D35" s="22" t="n"/>
-      <c r="E35" s="23" t="n"/>
-      <c r="F35" s="24" t="n"/>
+      <c r="B35" s="12" t="n"/>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="15" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="25" t="n">
+      <c r="A36" s="16" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="26" t="n"/>
-      <c r="C36" s="26" t="n"/>
-      <c r="D36" s="27" t="n"/>
-      <c r="E36" s="28" t="n"/>
-      <c r="F36" s="29" t="n"/>
+      <c r="B36" s="17" t="n"/>
+      <c r="C36" s="17" t="n"/>
+      <c r="D36" s="18" t="n"/>
+      <c r="E36" s="19" t="n"/>
+      <c r="F36" s="20" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="20" t="n">
+      <c r="A37" s="11" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="21" t="n"/>
-      <c r="C37" s="21" t="n"/>
-      <c r="D37" s="22" t="n"/>
-      <c r="E37" s="23" t="n"/>
-      <c r="F37" s="24" t="n"/>
+      <c r="B37" s="12" t="n"/>
+      <c r="C37" s="12" t="n"/>
+      <c r="D37" s="13" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="15" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="25" t="n">
+      <c r="A38" s="16" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="26" t="n"/>
-      <c r="C38" s="26" t="n"/>
-      <c r="D38" s="27" t="n"/>
-      <c r="E38" s="28" t="n"/>
-      <c r="F38" s="29" t="n"/>
+      <c r="B38" s="17" t="n"/>
+      <c r="C38" s="17" t="n"/>
+      <c r="D38" s="18" t="n"/>
+      <c r="E38" s="19" t="n"/>
+      <c r="F38" s="20" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="20" t="n">
+      <c r="A39" s="11" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="21" t="n"/>
-      <c r="C39" s="21" t="n"/>
-      <c r="D39" s="22" t="n"/>
-      <c r="E39" s="23" t="n"/>
-      <c r="F39" s="24" t="n"/>
+      <c r="B39" s="12" t="n"/>
+      <c r="C39" s="12" t="n"/>
+      <c r="D39" s="13" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="15" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
@@ -1362,119 +1249,119 @@
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ENTRAÎNEURS &amp; ACCOMPAGNATEURS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="17" t="n"/>
+      <c r="A2" s="8" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>2 accompagnateurs par équipe sont inclus dans les frais d'inscription (lignes 1 et 2). Les suivants sont facturés 40 € chacun et comptabilisés automatiquement dans l'onglet Accueil. Maximum 7 accompagnateurs.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Nom</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Prénom</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Email (obligatoire pour entraîneur)</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Rôle</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>1 ✓</t>
         </is>
       </c>
-      <c r="B5" s="32" t="n"/>
-      <c r="C5" s="32" t="n"/>
-      <c r="D5" s="32" t="n"/>
-      <c r="E5" s="33" t="n"/>
+      <c r="B5" s="23" t="n"/>
+      <c r="C5" s="23" t="n"/>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="24" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>2 ✓</t>
         </is>
       </c>
-      <c r="B6" s="32" t="n"/>
-      <c r="C6" s="32" t="n"/>
-      <c r="D6" s="32" t="n"/>
-      <c r="E6" s="33" t="n"/>
+      <c r="B6" s="23" t="n"/>
+      <c r="C6" s="23" t="n"/>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="24" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="20" t="n">
+      <c r="A7" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="21" t="n"/>
-      <c r="C7" s="21" t="n"/>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="34" t="n"/>
+      <c r="B7" s="12" t="n"/>
+      <c r="C7" s="12" t="n"/>
+      <c r="D7" s="12" t="n"/>
+      <c r="E7" s="25" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="25" t="n">
+      <c r="A8" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="26" t="n"/>
-      <c r="C8" s="26" t="n"/>
-      <c r="D8" s="26" t="n"/>
-      <c r="E8" s="35" t="n"/>
+      <c r="B8" s="17" t="n"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="26" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="20" t="n">
+      <c r="A9" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="21" t="n"/>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="34" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="25" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="25" t="n">
+      <c r="A10" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="26" t="n"/>
-      <c r="D10" s="26" t="n"/>
-      <c r="E10" s="35" t="n"/>
+      <c r="B10" s="17" t="n"/>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="26" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="20" t="n">
+      <c r="A11" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="21" t="n"/>
-      <c r="C11" s="21" t="n"/>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="34" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="25" t="n"/>
     </row>
     <row r="12" ht="10" customHeight="1"/>
     <row r="13" ht="50" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>RAPPEL RÈGLEMENT : Seuls les accompagnateurs et athlètes déclarés sont autorisés en salle d'échauffement et dans les vestiaires. Les accompagnateurs doivent arriver en même temps que leur équipe et se présenter à l'accueil pour récupérer leur bracelet.</t>
         </is>
@@ -1500,6 +1387,156 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00A0820A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>RÉSUMÉ &amp; CALCUL DES FRAIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="8" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>⚠ Les calculs ci-dessous sont automatiques et se mettent à jour en remplissant la feuille. Ne pas modifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="10" customHeight="1"/>
+    <row r="5" ht="22" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Nombre total d'athlètes</t>
+        </is>
+      </c>
+      <c r="C5" s="29">
+        <f>COUNTA(Athlètes!B5:B39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Dont athlètes masculins</t>
+        </is>
+      </c>
+      <c r="C6" s="29">
+        <f>COUNTIF(Athlètes!E5:E39,"M")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Accompagnateurs inclus (2/équipe)</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Accompagnateurs supplémentaires</t>
+        </is>
+      </c>
+      <c r="C8" s="29">
+        <f>MAX(0,COUNTA(Accompagnateurs!B5:B11)-2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Coût accompagnateurs suppl. (€)</t>
+        </is>
+      </c>
+      <c r="C9" s="30">
+        <f>C8*40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="10" customHeight="1"/>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Prix par athlète (€)</t>
+        </is>
+      </c>
+      <c r="C11" s="32">
+        <f>IF(Accueil!C8="Démo",35,IF(ISNUMBER(SEARCH("Allstar",Accueil!C8)),40,IF(OR(ISNUMBER(SEARCH("Prep",Accueil!C8)),ISNUMBER(SEARCH("Universitaire",Accueil!C8))),37.5,IF(Accueil!C8&lt;&gt;"","?",""))))</f>
+        <v/>
+      </c>
+      <c r="D11" s="33">
+        <f>IF(Accueil!C8="Démo","Démo : 35 €",IF(ISNUMBER(SEARCH("Allstar",Accueil!C8)),"Allstar : 40 €",IF(OR(ISNUMBER(SEARCH("Prep",Accueil!C8)),ISNUMBER(SEARCH("Universitaire",Accueil!C8))),"Universitaire / Prep : 37,50 €",IF(Accueil!C8&lt;&gt;"","? €","← sélectionnez une division"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="10" customHeight="1"/>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TOTAL ESTIMÉ (athlètes + accomp. suppl.)</t>
+        </is>
+      </c>
+      <c r="C13" s="35">
+        <f>C5*C11+C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="10" customHeight="1"/>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="36" t="inlineStr">
+        <is>
+          <t>Ce document ne fait pas office de facture. Les tarifs affichés sur le site crown-cheerleading-events.fr font valeur de référence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>Un acompte de 30 % est requis à l'inscription. Toute annulation avant la fermeture des inscriptions donne droit à un remboursement de 70 %, les 30 % d'acompte restant acquis. Le formulaire d'inscription pour l'envoi de ce fichier sera accessible à partir du 10 septembre 2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
+  <mergeCells count="8">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="D11:G11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>